<commit_message>
Entrega final verificada (auditoría adversarial de despieces)
Verificación exhaustiva de los 3 modelos (cargar_anotado + shapely, council adversarial):
- Validación limpia: Cabernet/Merlot/Chardonnay → 0 huecos, 0 solapes, 0 piezas en muro, área cuadra.
- PA-M-012/PA-M-020 (Chardonnay): el corte es MURO real (+ tira de cancelería 1 cm del DWG); completa=False correcto, NO es error.
- 'Arriba de PA-M-032' (Chardonnay): la franja está 99.8% dentro del muro #20 → correctamente sin enlosar, NO falta recorte.
- Notas de dibujo (severidad baja, NO alteran conteo): astillas de ~1 cm (PA-M-020/PB-M-133/PA-M-037) y baldosas sobredimensionadas PB-M-022/023 (1.21 m). No se corrigen en pipeline porque el fix rompía validación/geometría; quedan documentadas.
- Sin cambios de geometría: deliverables regenerados desde el pipeline validado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Generadores.xlsx
+++ b/Viñas Norte - Generadores.xlsx
@@ -702,7 +702,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    27/06/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    30/06/2026</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    27/06/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    30/06/2026</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    27/06/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    30/06/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chardonnay: quita la astilla de cancelería de 1 cm en PA-M-012 y PA-M-020
- _mascara_muros: resta las cajas de la nueva clave por-modelo 'cancel_ignorar' (tiras
  de cancelería de ~1 cm no serruchables) para que no aparezcan como notch.
- modelos.py Chardonnay: cancel_ignorar en x≈290.19-290.24 (columna A-CANCELERIA).
- Efecto (verificado por council en worktrees, enfoque B): SOLO cambian PA-M-012 y
  PA-M-020; conservan su recorte de MURO real (completa=False, notch limpio lado 0.12);
  se elimina el slot de 1 cm. Cabernet/Merlot intactos (cfg.get -> []).
- Validación limpia en los 3 (0 huecos/solapes/en_muro). Chardonnay área 154.10->154.12.
- Deliverables + ZIP regenerados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Generadores.xlsx
+++ b/Viñas Norte - Generadores.xlsx
@@ -702,7 +702,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    30/06/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    01/07/2026</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    30/06/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    01/07/2026</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    30/06/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    01/07/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
L19 M7 renivelado (digitalización verificada vs fotos nuevas) + despieces sin capa morada, sobrantes etiquetados y resumen de conteos
- Renivelación L19 M7 (Chardonnay): ambas plantas a RENIVELADO (2 de julio);
  f9 re-transcrito del plano impreso (73 puntos, escalera, fila 2,1,2,0,-1
  recuperada) y f8 corregido (7 valores, 17 puntos faltantes, reubicaciones);
  fotos nuevas en el PDF; totales 12.17 ejecutado / 3.87 por renivelar.
- Despieces (obs. de supervisión): se elimina la capa morada SOBRANTES-MAPA
  (tablones imaginarios encimados) del DXF y la página equivalente del PDF;
  cada sobrante amarillo lleva medida y destino (GUARDAR EN RESERVA); los
  recortes que salen de sobrante lo indican; cuadro RESUMEN en DXF con piezas
  completas / tablas abiertas / total / cajas y % de sobra, igual que el PDF.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Generadores.xlsx
+++ b/Viñas Norte - Generadores.xlsx
@@ -702,7 +702,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    01/07/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    03/07/2026</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    01/07/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    03/07/2026</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    01/07/2026</t>
+          <t>Elaboró: Ing. Mauricio Gastelum Mora    ·    03/07/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Detalles finales: fuera pieza en muro (Cabernet), recorte en L unificado (Chardonnay), zoclo del PDF bajo las etiquetas
- Cabernet: eliminada la pieza de umbral bajo PB-M-015 (esa franja es MURO,
  confirmado por el usuario; se revierte piezas_extra y la apertura de la
  mascara).
- Chardonnay: PB-M-069 + PB-M-073 unificadas en UN solo recorte en L
  (0.60 x 0.374 con el murete como entrante), en PDF y AutoCAD.
- PDF (pagina del plano): la linea de zoclo va DEBAJO de las etiquetas de
  pieza (zorder menor, mas delgada y translucida): ya no tapa textos en el
  Royal.
- Re-verificado: juntas exactas (787/788/785, 0 malas), 0 solapes, 0
  invasiones, 0 colinealidad rota, conteos QSELECT exactos en los 6 DXF.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Generadores.xlsx
+++ b/Viñas Norte - Generadores.xlsx
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>155.32</v>
+        <v>155.21</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>5.48</v>
+        <v>5.59</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>3.51</v>
@@ -1069,13 +1069,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>175.46</v>
+        <v>175.54</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>12.07</v>
+        <v>12.75</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>3.69</v>
+        <v>3.65</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>143</v>

</xml_diff>